<commit_message>
Search Vulnerabilities in new project
</commit_message>
<xml_diff>
--- a/resources/annotated_java_test.xlsx
+++ b/resources/annotated_java_test.xlsx
@@ -124,13 +124,13 @@
     <t>http://www.github.com/apache/shiro</t>
   </si>
   <si>
+    <t/>
+  </si>
+  <si>
+    <t>Security</t>
+  </si>
+  <si>
     <t>Mirror of Apache Shiro</t>
-  </si>
-  <si>
-    <t/>
-  </si>
-  <si>
-    <t>Security</t>
   </si>
 </sst>
 </file>
@@ -211,7 +211,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="13">
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0"/>
     <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -248,9 +248,6 @@
     </xf>
     <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
       <alignment horizontal="right"/>
-    </xf>
-    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
-      <alignment horizontal="general"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -577,8 +574,8 @@
     <col min="18" max="18" style="12" width="8.005" customWidth="1" bestFit="1"/>
     <col min="19" max="19" style="10" width="44.005" customWidth="1" bestFit="1"/>
     <col min="20" max="20" style="10" width="9.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="21" max="21" style="13" width="13.005" customWidth="1" bestFit="1"/>
-    <col min="22" max="22" style="13" width="18.005" customWidth="1" bestFit="1"/>
+    <col min="21" max="21" style="10" width="13.005" customWidth="1" bestFit="1"/>
+    <col min="22" max="22" style="10" width="18.005" customWidth="1" bestFit="1"/>
     <col min="23" max="23" style="10" width="94.86214285714286" customWidth="1" bestFit="1"/>
   </cols>
   <sheetData>
@@ -781,12 +778,12 @@
         <v>34</v>
       </c>
       <c r="T3" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="U3" s="9" t="s">
         <v>35</v>
       </c>
-      <c r="U3" s="4" t="s">
-        <v>28</v>
-      </c>
-      <c r="V3" s="9" t="s">
+      <c r="V3" s="4" t="s">
         <v>36</v>
       </c>
       <c r="W3" s="4" t="s">

</xml_diff>